<commit_message>
updating the screenshot for all questions
</commit_message>
<xml_diff>
--- a/SAP-C03/SAP-C02-ExamTopics-Questions.xlsx
+++ b/SAP-C03/SAP-C02-ExamTopics-Questions.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jetstarairways-my.sharepoint.com/personal/balraj_singh_jetstar_com/Documents/Balraj_D_Laptop_Drive/DevOps_Master/AWS-Exam-Certificate-Preparation/SAP-C03/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1157" documentId="8_{6D7FEDCE-BF68-490E-8FEE-13CF0653E58D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D415B8D-4240-4E53-B0CC-0E374B077870}"/>
+  <xr:revisionPtr revIDLastSave="1237" documentId="8_{6D7FEDCE-BF68-490E-8FEE-13CF0653E58D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{942BFD94-C0E5-4B4E-8359-F2E487A90595}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D730D107-BEC6-4E62-9FED-4CE422768F8C}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{D730D107-BEC6-4E62-9FED-4CE422768F8C}"/>
   </bookViews>
   <sheets>
-    <sheet name="ExamTopics" sheetId="4" r:id="rId1"/>
+    <sheet name="ExamTopics" sheetId="4" state="hidden" r:id="rId1"/>
     <sheet name="ExamTopics (SAP-C02)" sheetId="5" r:id="rId2"/>
   </sheets>
   <definedNames>
@@ -1759,7 +1759,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1785,6 +1785,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -7105,7 +7106,7 @@
       <c r="A452" s="1">
         <v>450</v>
       </c>
-      <c r="B452" t="s">
+      <c r="B452" s="9" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7113,7 +7114,7 @@
       <c r="A453" s="1">
         <v>451</v>
       </c>
-      <c r="B453" t="s">
+      <c r="B453" s="9" t="s">
         <v>53</v>
       </c>
     </row>
@@ -7121,7 +7122,7 @@
       <c r="A454" s="1">
         <v>452</v>
       </c>
-      <c r="B454" t="s">
+      <c r="B454" s="9" t="s">
         <v>502</v>
       </c>
     </row>
@@ -7129,7 +7130,7 @@
       <c r="A455" s="1">
         <v>453</v>
       </c>
-      <c r="B455" t="s">
+      <c r="B455" s="9" t="s">
         <v>34</v>
       </c>
     </row>
@@ -7137,7 +7138,7 @@
       <c r="A456" s="1">
         <v>454</v>
       </c>
-      <c r="B456" t="s">
+      <c r="B456" s="9" t="s">
         <v>52</v>
       </c>
     </row>
@@ -7145,7 +7146,7 @@
       <c r="A457" s="1">
         <v>455</v>
       </c>
-      <c r="B457" t="s">
+      <c r="B457" s="9" t="s">
         <v>297</v>
       </c>
     </row>
@@ -7153,7 +7154,7 @@
       <c r="A458" s="1">
         <v>456</v>
       </c>
-      <c r="B458" t="s">
+      <c r="B458" s="9" t="s">
         <v>445</v>
       </c>
     </row>
@@ -7161,7 +7162,7 @@
       <c r="A459" s="1">
         <v>457</v>
       </c>
-      <c r="B459" t="s">
+      <c r="B459" s="9" t="s">
         <v>430</v>
       </c>
     </row>
@@ -7169,7 +7170,7 @@
       <c r="A460" s="1">
         <v>458</v>
       </c>
-      <c r="B460" t="s">
+      <c r="B460" s="9" t="s">
         <v>309</v>
       </c>
     </row>
@@ -7177,7 +7178,7 @@
       <c r="A461" s="1">
         <v>459</v>
       </c>
-      <c r="B461" t="s">
+      <c r="B461" s="9" t="s">
         <v>464</v>
       </c>
     </row>
@@ -7185,7 +7186,7 @@
       <c r="A462" s="1">
         <v>460</v>
       </c>
-      <c r="B462" t="s">
+      <c r="B462" s="9" t="s">
         <v>444</v>
       </c>
     </row>
@@ -7193,7 +7194,7 @@
       <c r="A463" s="1">
         <v>461</v>
       </c>
-      <c r="B463" t="s">
+      <c r="B463" s="9" t="s">
         <v>51</v>
       </c>
     </row>
@@ -7201,7 +7202,7 @@
       <c r="A464" s="1">
         <v>462</v>
       </c>
-      <c r="B464" t="s">
+      <c r="B464" s="9" t="s">
         <v>424</v>
       </c>
     </row>
@@ -7209,7 +7210,7 @@
       <c r="A465" s="1">
         <v>463</v>
       </c>
-      <c r="B465" t="s">
+      <c r="B465" s="9" t="s">
         <v>495</v>
       </c>
     </row>
@@ -7217,7 +7218,7 @@
       <c r="A466" s="1">
         <v>464</v>
       </c>
-      <c r="B466" t="s">
+      <c r="B466" s="9" t="s">
         <v>401</v>
       </c>
     </row>
@@ -7225,7 +7226,7 @@
       <c r="A467" s="1">
         <v>465</v>
       </c>
-      <c r="B467" t="s">
+      <c r="B467" s="9" t="s">
         <v>443</v>
       </c>
     </row>
@@ -7233,7 +7234,7 @@
       <c r="A468" s="1">
         <v>466</v>
       </c>
-      <c r="B468" t="s">
+      <c r="B468" s="9" t="s">
         <v>505</v>
       </c>
     </row>
@@ -7241,7 +7242,7 @@
       <c r="A469" s="1">
         <v>467</v>
       </c>
-      <c r="B469" t="s">
+      <c r="B469" s="9" t="s">
         <v>33</v>
       </c>
     </row>
@@ -7249,7 +7250,7 @@
       <c r="A470" s="1">
         <v>468</v>
       </c>
-      <c r="B470" t="s">
+      <c r="B470" s="9" t="s">
         <v>442</v>
       </c>
     </row>
@@ -7257,7 +7258,7 @@
       <c r="A471" s="1">
         <v>469</v>
       </c>
-      <c r="B471" t="s">
+      <c r="B471" s="9" t="s">
         <v>441</v>
       </c>
     </row>
@@ -7265,7 +7266,7 @@
       <c r="A472" s="1">
         <v>470</v>
       </c>
-      <c r="B472" t="s">
+      <c r="B472" s="9" t="s">
         <v>136</v>
       </c>
     </row>
@@ -7273,7 +7274,7 @@
       <c r="A473" s="1">
         <v>471</v>
       </c>
-      <c r="B473" t="s">
+      <c r="B473" s="9" t="s">
         <v>32</v>
       </c>
     </row>
@@ -7281,7 +7282,7 @@
       <c r="A474" s="1">
         <v>472</v>
       </c>
-      <c r="B474" t="s">
+      <c r="B474" s="9" t="s">
         <v>128</v>
       </c>
     </row>
@@ -7289,7 +7290,7 @@
       <c r="A475" s="1">
         <v>473</v>
       </c>
-      <c r="B475" t="s">
+      <c r="B475" s="9" t="s">
         <v>335</v>
       </c>
     </row>
@@ -7297,7 +7298,7 @@
       <c r="A476" s="1">
         <v>474</v>
       </c>
-      <c r="B476" t="s">
+      <c r="B476" s="9" t="s">
         <v>215</v>
       </c>
     </row>
@@ -7305,7 +7306,7 @@
       <c r="A477" s="1">
         <v>475</v>
       </c>
-      <c r="B477" t="s">
+      <c r="B477" s="9" t="s">
         <v>417</v>
       </c>
     </row>
@@ -7313,7 +7314,7 @@
       <c r="A478" s="1">
         <v>476</v>
       </c>
-      <c r="B478" t="s">
+      <c r="B478" s="9" t="s">
         <v>204</v>
       </c>
     </row>
@@ -7321,7 +7322,7 @@
       <c r="A479" s="1">
         <v>477</v>
       </c>
-      <c r="B479" t="s">
+      <c r="B479" s="9" t="s">
         <v>510</v>
       </c>
     </row>
@@ -7329,7 +7330,7 @@
       <c r="A480" s="1">
         <v>478</v>
       </c>
-      <c r="B480" t="s">
+      <c r="B480" s="9" t="s">
         <v>439</v>
       </c>
     </row>
@@ -7337,7 +7338,7 @@
       <c r="A481" s="1">
         <v>479</v>
       </c>
-      <c r="B481" t="s">
+      <c r="B481" s="9" t="s">
         <v>146</v>
       </c>
     </row>
@@ -7345,7 +7346,7 @@
       <c r="A482" s="1">
         <v>480</v>
       </c>
-      <c r="B482" t="s">
+      <c r="B482" s="9" t="s">
         <v>77</v>
       </c>
     </row>
@@ -7353,7 +7354,7 @@
       <c r="A483" s="1">
         <v>481</v>
       </c>
-      <c r="B483" t="s">
+      <c r="B483" s="9" t="s">
         <v>465</v>
       </c>
     </row>
@@ -7361,7 +7362,7 @@
       <c r="A484" s="1">
         <v>482</v>
       </c>
-      <c r="B484" t="s">
+      <c r="B484" s="9" t="s">
         <v>438</v>
       </c>
     </row>
@@ -7369,7 +7370,7 @@
       <c r="A485" s="1">
         <v>483</v>
       </c>
-      <c r="B485" t="s">
+      <c r="B485" s="9" t="s">
         <v>153</v>
       </c>
     </row>
@@ -7377,7 +7378,7 @@
       <c r="A486" s="1">
         <v>484</v>
       </c>
-      <c r="B486" t="s">
+      <c r="B486" s="9" t="s">
         <v>425</v>
       </c>
     </row>
@@ -7385,7 +7386,7 @@
       <c r="A487" s="1">
         <v>485</v>
       </c>
-      <c r="B487" t="s">
+      <c r="B487" s="9" t="s">
         <v>468</v>
       </c>
     </row>
@@ -7393,7 +7394,7 @@
       <c r="A488" s="1">
         <v>486</v>
       </c>
-      <c r="B488" t="s">
+      <c r="B488" s="9" t="s">
         <v>397</v>
       </c>
     </row>
@@ -7401,7 +7402,7 @@
       <c r="A489" s="1">
         <v>487</v>
       </c>
-      <c r="B489" t="s">
+      <c r="B489" s="9" t="s">
         <v>29</v>
       </c>
     </row>
@@ -7409,7 +7410,7 @@
       <c r="A490" s="1">
         <v>488</v>
       </c>
-      <c r="B490" t="s">
+      <c r="B490" s="9" t="s">
         <v>474</v>
       </c>
     </row>
@@ -7417,7 +7418,7 @@
       <c r="A491" s="1">
         <v>489</v>
       </c>
-      <c r="B491" t="s">
+      <c r="B491" s="9" t="s">
         <v>400</v>
       </c>
     </row>
@@ -7425,7 +7426,7 @@
       <c r="A492" s="1">
         <v>490</v>
       </c>
-      <c r="B492" t="s">
+      <c r="B492" s="9" t="s">
         <v>426</v>
       </c>
     </row>
@@ -7433,7 +7434,7 @@
       <c r="A493" s="1">
         <v>491</v>
       </c>
-      <c r="B493" t="s">
+      <c r="B493" s="9" t="s">
         <v>345</v>
       </c>
     </row>
@@ -7441,7 +7442,7 @@
       <c r="A494" s="1">
         <v>492</v>
       </c>
-      <c r="B494" t="s">
+      <c r="B494" s="9" t="s">
         <v>344</v>
       </c>
     </row>
@@ -7449,7 +7450,7 @@
       <c r="A495" s="1">
         <v>493</v>
       </c>
-      <c r="B495" t="s">
+      <c r="B495" s="9" t="s">
         <v>343</v>
       </c>
     </row>
@@ -7457,7 +7458,7 @@
       <c r="A496" s="1">
         <v>494</v>
       </c>
-      <c r="B496" t="s">
+      <c r="B496" s="9" t="s">
         <v>383</v>
       </c>
     </row>
@@ -7465,7 +7466,7 @@
       <c r="A497" s="1">
         <v>495</v>
       </c>
-      <c r="B497" t="s">
+      <c r="B497" s="9" t="s">
         <v>382</v>
       </c>
     </row>
@@ -7473,7 +7474,7 @@
       <c r="A498" s="1">
         <v>496</v>
       </c>
-      <c r="B498" t="s">
+      <c r="B498" s="9" t="s">
         <v>392</v>
       </c>
     </row>
@@ -7481,7 +7482,7 @@
       <c r="A499" s="1">
         <v>497</v>
       </c>
-      <c r="B499" t="s">
+      <c r="B499" s="9" t="s">
         <v>507</v>
       </c>
     </row>
@@ -7489,7 +7490,7 @@
       <c r="A500" s="1">
         <v>498</v>
       </c>
-      <c r="B500" t="s">
+      <c r="B500" s="9" t="s">
         <v>407</v>
       </c>
     </row>
@@ -7497,7 +7498,7 @@
       <c r="A501" s="1">
         <v>499</v>
       </c>
-      <c r="B501" t="s">
+      <c r="B501" s="9" t="s">
         <v>418</v>
       </c>
     </row>
@@ -7505,7 +7506,7 @@
       <c r="A502" s="1">
         <v>500</v>
       </c>
-      <c r="B502" t="s">
+      <c r="B502" s="9" t="s">
         <v>166</v>
       </c>
     </row>
@@ -7513,7 +7514,7 @@
       <c r="A503" s="1">
         <v>501</v>
       </c>
-      <c r="B503" t="s">
+      <c r="B503" s="9" t="s">
         <v>54</v>
       </c>
     </row>
@@ -7521,7 +7522,7 @@
       <c r="A504" s="1">
         <v>502</v>
       </c>
-      <c r="B504" t="s">
+      <c r="B504" s="9" t="s">
         <v>342</v>
       </c>
     </row>
@@ -7529,7 +7530,7 @@
       <c r="A505" s="1">
         <v>503</v>
       </c>
-      <c r="B505" t="s">
+      <c r="B505" s="9" t="s">
         <v>55</v>
       </c>
     </row>
@@ -7537,7 +7538,7 @@
       <c r="A506" s="1">
         <v>504</v>
       </c>
-      <c r="B506" t="s">
+      <c r="B506" s="9" t="s">
         <v>393</v>
       </c>
     </row>
@@ -7545,7 +7546,7 @@
       <c r="A507" s="1">
         <v>505</v>
       </c>
-      <c r="B507" t="s">
+      <c r="B507" s="9" t="s">
         <v>521</v>
       </c>
     </row>
@@ -7553,7 +7554,7 @@
       <c r="A508" s="1">
         <v>506</v>
       </c>
-      <c r="B508" t="s">
+      <c r="B508" s="9" t="s">
         <v>56</v>
       </c>
     </row>
@@ -7561,7 +7562,7 @@
       <c r="A509" s="1">
         <v>507</v>
       </c>
-      <c r="B509" t="s">
+      <c r="B509" s="9" t="s">
         <v>135</v>
       </c>
     </row>
@@ -7569,7 +7570,7 @@
       <c r="A510" s="1">
         <v>508</v>
       </c>
-      <c r="B510" t="s">
+      <c r="B510" s="9" t="s">
         <v>57</v>
       </c>
     </row>
@@ -7577,7 +7578,7 @@
       <c r="A511" s="1">
         <v>509</v>
       </c>
-      <c r="B511" t="s">
+      <c r="B511" s="9" t="s">
         <v>311</v>
       </c>
     </row>
@@ -7585,7 +7586,7 @@
       <c r="A512" s="1">
         <v>510</v>
       </c>
-      <c r="B512" t="s">
+      <c r="B512" s="9" t="s">
         <v>207</v>
       </c>
     </row>
@@ -7593,7 +7594,7 @@
       <c r="A513" s="1">
         <v>511</v>
       </c>
-      <c r="B513" t="s">
+      <c r="B513" s="9" t="s">
         <v>330</v>
       </c>
     </row>
@@ -7601,7 +7602,7 @@
       <c r="A514" s="1">
         <v>512</v>
       </c>
-      <c r="B514" t="s">
+      <c r="B514" s="9" t="s">
         <v>84</v>
       </c>
     </row>
@@ -7609,7 +7610,7 @@
       <c r="A515" s="1">
         <v>513</v>
       </c>
-      <c r="B515" t="s">
+      <c r="B515" s="9" t="s">
         <v>497</v>
       </c>
     </row>
@@ -7617,7 +7618,7 @@
       <c r="A516" s="1">
         <v>514</v>
       </c>
-      <c r="B516" t="s">
+      <c r="B516" s="9" t="s">
         <v>45</v>
       </c>
     </row>
@@ -7625,7 +7626,7 @@
       <c r="A517" s="1">
         <v>515</v>
       </c>
-      <c r="B517" t="s">
+      <c r="B517" s="9" t="s">
         <v>58</v>
       </c>
     </row>
@@ -7633,7 +7634,7 @@
       <c r="A518" s="1">
         <v>516</v>
       </c>
-      <c r="B518" t="s">
+      <c r="B518" s="9" t="s">
         <v>353</v>
       </c>
     </row>
@@ -7641,7 +7642,7 @@
       <c r="A519" s="1">
         <v>517</v>
       </c>
-      <c r="B519" t="s">
+      <c r="B519" s="9" t="s">
         <v>380</v>
       </c>
     </row>
@@ -7649,7 +7650,7 @@
       <c r="A520" s="1">
         <v>518</v>
       </c>
-      <c r="B520" t="s">
+      <c r="B520" s="9" t="s">
         <v>403</v>
       </c>
     </row>
@@ -7657,7 +7658,7 @@
       <c r="A521" s="1">
         <v>519</v>
       </c>
-      <c r="B521" t="s">
+      <c r="B521" s="9" t="s">
         <v>432</v>
       </c>
     </row>
@@ -7665,7 +7666,7 @@
       <c r="A522" s="1">
         <v>520</v>
       </c>
-      <c r="B522" t="s">
+      <c r="B522" s="9" t="s">
         <v>508</v>
       </c>
     </row>
@@ -7673,7 +7674,7 @@
       <c r="A523" s="1">
         <v>521</v>
       </c>
-      <c r="B523" t="s">
+      <c r="B523" s="9" t="s">
         <v>408</v>
       </c>
     </row>
@@ -7681,7 +7682,7 @@
       <c r="A524" s="1">
         <v>522</v>
       </c>
-      <c r="B524" t="s">
+      <c r="B524" s="9" t="s">
         <v>341</v>
       </c>
     </row>
@@ -7689,7 +7690,7 @@
       <c r="A525" s="1">
         <v>523</v>
       </c>
-      <c r="B525" t="s">
+      <c r="B525" s="9" t="s">
         <v>376</v>
       </c>
     </row>
@@ -7697,7 +7698,7 @@
       <c r="A526" s="1">
         <v>524</v>
       </c>
-      <c r="B526" t="s">
+      <c r="B526" s="9" t="s">
         <v>312</v>
       </c>
     </row>
@@ -7705,7 +7706,7 @@
       <c r="A527" s="1">
         <v>525</v>
       </c>
-      <c r="B527" t="s">
+      <c r="B527" s="9" t="s">
         <v>148</v>
       </c>
     </row>
@@ -7713,7 +7714,7 @@
       <c r="A528" s="1">
         <v>526</v>
       </c>
-      <c r="B528" t="s">
+      <c r="B528" s="9" t="s">
         <v>220</v>
       </c>
     </row>
@@ -7721,7 +7722,7 @@
       <c r="A529" s="1">
         <v>527</v>
       </c>
-      <c r="B529" t="s">
+      <c r="B529" s="9" t="s">
         <v>59</v>
       </c>
     </row>
@@ -7729,7 +7730,7 @@
       <c r="A530" s="1">
         <v>528</v>
       </c>
-      <c r="B530" t="s">
+      <c r="B530" s="9" t="s">
         <v>375</v>
       </c>
     </row>
@@ -7737,7 +7738,7 @@
       <c r="A531" s="1">
         <v>529</v>
       </c>
-      <c r="B531" t="s">
+      <c r="B531" s="9" t="s">
         <v>49</v>
       </c>
     </row>
@@ -7750,5 +7751,6 @@
     <hyperlink ref="A1" r:id="rId1" xr:uid="{E4BE23F5-8686-4318-92B6-7D7B715CDD5E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>